<commit_message>
feat(remove lines and run case A)
Testing case A with IEEE 6 ww - Success
</commit_message>
<xml_diff>
--- a/01_Data/00_Templates/plantilla_datos.xlsx
+++ b/01_Data/00_Templates/plantilla_datos.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\My Drive\2. Universidad Nacional de Colombia\2. Postgraduate\1_SEMESTER\TESIS DE MAESTRIA\2nd Search\04_TESIS_DANIEL\03_CODIGO_TRABAJO_DANIEL\BESS_FACTS_master\01_Data\00_Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B8E067C-2DCC-493F-82FC-DC8084BE8E5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2823B3AF-7937-4530-893A-CA694B8EC43B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6945" yWindow="3270" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="INSTRUCCIONES" sheetId="1" r:id="rId1"/>
     <sheet name="Config" sheetId="2" r:id="rId2"/>
     <sheet name="Nodos" sheetId="3" r:id="rId3"/>
     <sheet name="Lineas" sheetId="4" r:id="rId4"/>
-    <sheet name="Lineas_Cand" sheetId="5" r:id="rId5"/>
+    <sheet name="Lineas_Cand" sheetId="5" state="hidden" r:id="rId5"/>
     <sheet name="Generadores" sheetId="6" r:id="rId6"/>
     <sheet name="Hidraulicos" sheetId="7" r:id="rId7"/>
     <sheet name="Renovables" sheetId="8" r:id="rId8"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="114">
   <si>
     <t>Plantilla de datos - Modelo TEP con BESS y FACTS</t>
   </si>
@@ -354,6 +354,24 @@
   </si>
   <si>
     <t>UNIDADES: indicadas en la fila bajo cada encabezado. (No borrarlas ni modificarlas)</t>
+  </si>
+  <si>
+    <t>vida_bess</t>
+  </si>
+  <si>
+    <t>vida_facts</t>
+  </si>
+  <si>
+    <t>años</t>
+  </si>
+  <si>
+    <t>años NREL</t>
+  </si>
+  <si>
+    <t>incluir_perdidas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0 (sin pérdidas - validación DC); 1(con pérdidas) </t>
   </si>
 </sst>
 </file>
@@ -438,7 +456,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -454,7 +472,16 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1124,7 +1151,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="44.42578125" bestFit="1" customWidth="1"/>
@@ -1189,7 +1216,7 @@
       <c r="A9" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B9" s="7"/>
+      <c r="B9" s="5"/>
       <c r="C9" s="6" t="s">
         <v>29</v>
       </c>
@@ -1198,7 +1225,7 @@
       <c r="A10" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="B10" s="7"/>
+      <c r="B10" s="5"/>
       <c r="C10" s="6" t="s">
         <v>31</v>
       </c>
@@ -1207,9 +1234,36 @@
       <c r="A11" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B11" s="7"/>
+      <c r="B11" s="5"/>
       <c r="C11" s="6" t="s">
         <v>33</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="B12" s="7"/>
+      <c r="C12" s="8" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="B13" s="7"/>
+      <c r="C13" s="8" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="B14" s="10"/>
+      <c r="C14" s="9" t="s">
+        <v>113</v>
       </c>
     </row>
   </sheetData>

</xml_diff>